<commit_message>
feat(investor): regroupement des projets CASTEBRUNET (4 stations BESS) et JARRY (2 hangars PV)
</commit_message>
<xml_diff>
--- a/public/documents/dataroom/Business_plans_unitaires_chronique_20_ans_HELIOS.xlsx
+++ b/public/documents/dataroom/Business_plans_unitaires_chronique_20_ans_HELIOS.xlsx
@@ -663,7 +663,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:K17"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -694,30 +694,24 @@
         <v>Dpt</v>
       </c>
       <c r="E1" t="str">
+        <v>Exploitant / Client</v>
+      </c>
+      <c r="F1" t="str">
         <v>Puissance (kWc)</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Surface Toiture (m²)</v>
       </c>
-      <c r="G1" t="str">
-        <v>Productible P50 (kWh/kWc)</v>
-      </c>
       <c r="H1" t="str">
-        <v>Production An 1 (kWh)</v>
+        <v>Coût Travaux HT (€)</v>
       </c>
       <c r="I1" t="str">
-        <v>Tarif S21 (€/MWh)</v>
+        <v>CA Brut An 1 (€ HT)</v>
       </c>
       <c r="J1" t="str">
-        <v>CA Brut An 1 (€ HT)</v>
+        <v>Statut Foncier</v>
       </c>
       <c r="K1" t="str">
-        <v>Loyer Foncier (€/an)</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Statut Foncier</v>
-      </c>
-      <c r="M1" t="str">
         <v>Statut Urba</v>
       </c>
     </row>
@@ -726,40 +720,34 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>CONSOLI</v>
+        <v>CONDOM</v>
       </c>
       <c r="C2" t="str">
-        <v>24130 PRIGONRIEUX</v>
+        <v>32100 CONDOM</v>
       </c>
       <c r="D2" t="str">
-        <v>24</v>
-      </c>
-      <c r="E2">
-        <v>498.4</v>
+        <v>32</v>
+      </c>
+      <c r="E2" t="str">
+        <v>SAINT ARAILLES Henri</v>
       </c>
       <c r="F2">
-        <v>2800</v>
+        <v>256</v>
       </c>
       <c r="G2">
-        <v>1130</v>
+        <v>1485</v>
       </c>
       <c r="H2">
-        <v>563192</v>
+        <v>164194</v>
       </c>
       <c r="I2">
-        <v>82</v>
-      </c>
-      <c r="J2">
-        <v>46182</v>
-      </c>
-      <c r="K2">
-        <v>3500</v>
-      </c>
-      <c r="L2" t="str">
+        <v>23347</v>
+      </c>
+      <c r="J2" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M2" t="str">
-        <v>URBA OK (DP purgée)</v>
+      <c r="K2" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="3">
@@ -767,40 +755,34 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>LABEGUERIE</v>
+        <v>BRANTÔME EN PÉRIGORD</v>
       </c>
       <c r="C3" t="str">
-        <v>64120 ORÈGUE</v>
+        <v>24310 BRANTÔME</v>
       </c>
       <c r="D3" t="str">
-        <v>64</v>
-      </c>
-      <c r="E3">
-        <v>500</v>
+        <v>24</v>
+      </c>
+      <c r="E3" t="str">
+        <v>LATOURNERIE Nicolas</v>
       </c>
       <c r="F3">
-        <v>2750</v>
+        <v>1006</v>
       </c>
       <c r="G3">
-        <v>1120</v>
+        <v>5835</v>
       </c>
       <c r="H3">
-        <v>560000</v>
+        <v>528619</v>
       </c>
       <c r="I3">
-        <v>82</v>
-      </c>
-      <c r="J3">
-        <v>45920</v>
-      </c>
-      <c r="K3">
-        <v>3500</v>
-      </c>
-      <c r="L3" t="str">
+        <v>92680</v>
+      </c>
+      <c r="J3" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M3" t="str">
-        <v>URBA OK (PC obtenu)</v>
+      <c r="K3" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="4">
@@ -808,40 +790,34 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>CHOLOUX</v>
+        <v>GARONS</v>
       </c>
       <c r="C4" t="str">
-        <v>16210 CHALAIS</v>
+        <v>30128 GARONS</v>
       </c>
       <c r="D4" t="str">
-        <v>16</v>
-      </c>
-      <c r="E4">
-        <v>360</v>
+        <v>30</v>
+      </c>
+      <c r="E4" t="str">
+        <v>RODIER-VARGAS Cécile</v>
       </c>
       <c r="F4">
-        <v>2100</v>
+        <v>460</v>
       </c>
       <c r="G4">
-        <v>1115</v>
+        <v>2668</v>
       </c>
       <c r="H4">
-        <v>401400</v>
+        <v>265154</v>
       </c>
       <c r="I4">
-        <v>82</v>
-      </c>
-      <c r="J4">
-        <v>32915</v>
-      </c>
-      <c r="K4">
-        <v>2800</v>
-      </c>
-      <c r="L4" t="str">
+        <v>41952</v>
+      </c>
+      <c r="J4" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M4" t="str">
-        <v>URBA OK (PC obtenu)</v>
+      <c r="K4" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="5">
@@ -849,40 +825,34 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>MISSAULT 1</v>
+        <v>VAL-DE-LIVENNE</v>
       </c>
       <c r="C5" t="str">
-        <v>24470 SAINT-SAUD</v>
+        <v>33860 VAL-DE-LIVENNE</v>
       </c>
       <c r="D5" t="str">
-        <v>24</v>
-      </c>
-      <c r="E5">
-        <v>450</v>
+        <v>33</v>
+      </c>
+      <c r="E5" t="str">
+        <v>HERIT Dominique</v>
       </c>
       <c r="F5">
-        <v>2500</v>
+        <v>120</v>
       </c>
       <c r="G5">
-        <v>1125</v>
+        <v>696</v>
       </c>
       <c r="H5">
-        <v>506250</v>
+        <v>96888</v>
       </c>
       <c r="I5">
-        <v>82</v>
-      </c>
-      <c r="J5">
-        <v>41513</v>
-      </c>
-      <c r="K5">
-        <v>3200</v>
-      </c>
-      <c r="L5" t="str">
+        <v>10944</v>
+      </c>
+      <c r="J5" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M5" t="str">
-        <v>URBA OK (DP purgée)</v>
+      <c r="K5" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="6">
@@ -890,40 +860,34 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>MISSAULT 2</v>
+        <v>LACQUY</v>
       </c>
       <c r="C6" t="str">
-        <v>24800 ST-MARTIN</v>
+        <v>40120 LACQUY</v>
       </c>
       <c r="D6" t="str">
-        <v>24</v>
-      </c>
-      <c r="E6">
-        <v>500</v>
+        <v>40</v>
+      </c>
+      <c r="E6" t="str">
+        <v>LECONTE Frédéric</v>
       </c>
       <c r="F6">
-        <v>2800</v>
+        <v>145</v>
       </c>
       <c r="G6">
-        <v>1125</v>
+        <v>841</v>
       </c>
       <c r="H6">
-        <v>562500</v>
+        <v>109261</v>
       </c>
       <c r="I6">
-        <v>82</v>
-      </c>
-      <c r="J6">
-        <v>46125</v>
-      </c>
-      <c r="K6">
-        <v>3500</v>
-      </c>
-      <c r="L6" t="str">
+        <v>13224</v>
+      </c>
+      <c r="J6" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M6" t="str">
-        <v>URBA OK (PC obtenu)</v>
+      <c r="K6" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="7">
@@ -931,40 +895,34 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>ARBOIN</v>
+        <v>PUYLAUSIC</v>
       </c>
       <c r="C7" t="str">
-        <v>47120 DURAS</v>
+        <v>32220 PUYLAUSIC</v>
       </c>
       <c r="D7" t="str">
-        <v>47</v>
-      </c>
-      <c r="E7">
-        <v>480</v>
+        <v>32</v>
+      </c>
+      <c r="E7" t="str">
+        <v>CASSAGNE Christian</v>
       </c>
       <c r="F7">
-        <v>2700</v>
+        <v>157</v>
       </c>
       <c r="G7">
-        <v>1140</v>
+        <v>911</v>
       </c>
       <c r="H7">
-        <v>547200</v>
+        <v>115199</v>
       </c>
       <c r="I7">
-        <v>82</v>
-      </c>
-      <c r="J7">
-        <v>44870</v>
-      </c>
-      <c r="K7">
-        <v>3400</v>
-      </c>
-      <c r="L7" t="str">
+        <v>14318</v>
+      </c>
+      <c r="J7" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M7" t="str">
-        <v>URBA OK (DP purgée)</v>
+      <c r="K7" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="8">
@@ -972,40 +930,34 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>BERTRANDIE</v>
+        <v>SAINT-LAURENT-DU-PLAN</v>
       </c>
       <c r="C8" t="str">
-        <v>24240 MONESTIER</v>
+        <v>33190 ST-LAURENT</v>
       </c>
       <c r="D8" t="str">
-        <v>24</v>
-      </c>
-      <c r="E8">
-        <v>420</v>
+        <v>33</v>
+      </c>
+      <c r="E8" t="str">
+        <v>LECONTE Frédéric</v>
       </c>
       <c r="F8">
-        <v>2400</v>
+        <v>485</v>
       </c>
       <c r="G8">
-        <v>1135</v>
+        <v>2813</v>
       </c>
       <c r="H8">
-        <v>476700</v>
+        <v>277527</v>
       </c>
       <c r="I8">
-        <v>82</v>
-      </c>
-      <c r="J8">
-        <v>39089</v>
-      </c>
-      <c r="K8">
-        <v>3000</v>
-      </c>
-      <c r="L8" t="str">
+        <v>44232</v>
+      </c>
+      <c r="J8" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M8" t="str">
-        <v>URBA OK (DP purgée)</v>
+      <c r="K8" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="9">
@@ -1013,40 +965,34 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>CASTEBRUNET 1</v>
+        <v>LECTOURE</v>
       </c>
       <c r="C9" t="str">
-        <v>82300 CAUSSADE</v>
+        <v>32700 LECTOURE</v>
       </c>
       <c r="D9" t="str">
-        <v>82</v>
-      </c>
-      <c r="E9">
-        <v>500</v>
+        <v>32</v>
+      </c>
+      <c r="E9" t="str">
+        <v>RECKINGER Nicolas</v>
       </c>
       <c r="F9">
-        <v>2800</v>
+        <v>789</v>
       </c>
       <c r="G9">
-        <v>1145</v>
+        <v>4576</v>
       </c>
       <c r="H9">
-        <v>572500</v>
+        <v>427976</v>
       </c>
       <c r="I9">
-        <v>82</v>
-      </c>
-      <c r="J9">
-        <v>46945</v>
-      </c>
-      <c r="K9">
-        <v>3500</v>
-      </c>
-      <c r="L9" t="str">
+        <v>71957</v>
+      </c>
+      <c r="J9" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M9" t="str">
-        <v>URBA OK (PC obtenu)</v>
+      <c r="K9" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="10">
@@ -1054,40 +1000,34 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>CASTEBRUNET 2</v>
+        <v>GORNAC (JARRY 1 &amp; JARRY 2)</v>
       </c>
       <c r="C10" t="str">
-        <v>82300 CAUSSADE</v>
+        <v>33540 GORNAC</v>
       </c>
       <c r="D10" t="str">
-        <v>82</v>
-      </c>
-      <c r="E10">
-        <v>360</v>
+        <v>33</v>
+      </c>
+      <c r="E10" t="str">
+        <v>JARRY Frédéric (Cluster 2 hangars)</v>
       </c>
       <c r="F10">
-        <v>2050</v>
+        <v>628</v>
       </c>
       <c r="G10">
-        <v>1145</v>
+        <v>3642</v>
       </c>
       <c r="H10">
-        <v>412200</v>
+        <v>348297</v>
       </c>
       <c r="I10">
-        <v>82</v>
-      </c>
-      <c r="J10">
-        <v>33800</v>
-      </c>
-      <c r="K10">
-        <v>2600</v>
-      </c>
-      <c r="L10" t="str">
+        <v>57274</v>
+      </c>
+      <c r="J10" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M10" t="str">
-        <v>URBA OK (PC obtenu)</v>
+      <c r="K10" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="11">
@@ -1095,40 +1035,34 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>DAVID</v>
+        <v>CHALAIS</v>
       </c>
       <c r="C11" t="str">
-        <v>19350 CONCÈZE</v>
+        <v>16210 CHALAIS</v>
       </c>
       <c r="D11" t="str">
-        <v>19</v>
-      </c>
-      <c r="E11">
-        <v>300</v>
+        <v>16</v>
+      </c>
+      <c r="E11" t="str">
+        <v>CHOLOUX Jean-Marc</v>
       </c>
       <c r="F11">
-        <v>1750</v>
+        <v>707.2</v>
       </c>
       <c r="G11">
-        <v>1110</v>
+        <v>4102</v>
       </c>
       <c r="H11">
-        <v>333000</v>
+        <v>387493</v>
       </c>
       <c r="I11">
-        <v>82</v>
-      </c>
-      <c r="J11">
-        <v>27306</v>
-      </c>
-      <c r="K11">
-        <v>2200</v>
-      </c>
-      <c r="L11" t="str">
+        <v>64497</v>
+      </c>
+      <c r="J11" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M11" t="str">
-        <v>URBA OK (DP purgée)</v>
+      <c r="K11" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="12">
@@ -1136,40 +1070,34 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>DOMERGUE</v>
+        <v>MIRAMBEAU</v>
       </c>
       <c r="C12" t="str">
-        <v>87380 MEUZAC</v>
+        <v>17150 MIRAMBEAU</v>
       </c>
       <c r="D12" t="str">
-        <v>87</v>
-      </c>
-      <c r="E12">
-        <v>450</v>
+        <v>17</v>
+      </c>
+      <c r="E12" t="str">
+        <v>CHAUCHET Eric</v>
       </c>
       <c r="F12">
-        <v>2550</v>
+        <v>145</v>
       </c>
       <c r="G12">
-        <v>1105</v>
+        <v>841</v>
       </c>
       <c r="H12">
-        <v>497250</v>
+        <v>109261</v>
       </c>
       <c r="I12">
-        <v>82</v>
-      </c>
-      <c r="J12">
-        <v>40775</v>
-      </c>
-      <c r="K12">
-        <v>3200</v>
-      </c>
-      <c r="L12" t="str">
+        <v>13224</v>
+      </c>
+      <c r="J12" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M12" t="str">
-        <v>URBA OK (DP purgée)</v>
+      <c r="K12" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="13">
@@ -1177,40 +1105,34 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>DOUMENS</v>
+        <v>SAINT-SAUD-LACOUSSIÈRE</v>
       </c>
       <c r="C13" t="str">
-        <v>33750 BEYCHAC</v>
+        <v>24470 ST-SAUD</v>
       </c>
       <c r="D13" t="str">
-        <v>33</v>
-      </c>
-      <c r="E13">
-        <v>420</v>
+        <v>24</v>
+      </c>
+      <c r="E13" t="str">
+        <v>MISSAULT Patrick</v>
       </c>
       <c r="F13">
-        <v>2350</v>
+        <v>434</v>
       </c>
       <c r="G13">
-        <v>1130</v>
+        <v>2517</v>
       </c>
       <c r="H13">
-        <v>474600</v>
+        <v>279787</v>
       </c>
       <c r="I13">
-        <v>82</v>
-      </c>
-      <c r="J13">
-        <v>38917</v>
-      </c>
-      <c r="K13">
-        <v>3000</v>
-      </c>
-      <c r="L13" t="str">
+        <v>39407</v>
+      </c>
+      <c r="J13" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M13" t="str">
-        <v>URBA OK (PC obtenu)</v>
+      <c r="K13" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="14">
@@ -1218,40 +1140,34 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>GIOT</v>
+        <v>JUSSAS</v>
       </c>
       <c r="C14" t="str">
-        <v>23600 LEYRAT</v>
+        <v>17130 JUSSAS</v>
       </c>
       <c r="D14" t="str">
-        <v>23</v>
-      </c>
-      <c r="E14">
-        <v>380</v>
+        <v>17</v>
+      </c>
+      <c r="E14" t="str">
+        <v>DUHARD Christian</v>
       </c>
       <c r="F14">
-        <v>2150</v>
+        <v>181</v>
       </c>
       <c r="G14">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="H14">
-        <v>418000</v>
+        <v>127077</v>
       </c>
       <c r="I14">
-        <v>82</v>
-      </c>
-      <c r="J14">
-        <v>34276</v>
-      </c>
-      <c r="K14">
-        <v>2700</v>
-      </c>
-      <c r="L14" t="str">
+        <v>16507</v>
+      </c>
+      <c r="J14" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M14" t="str">
-        <v>URBA OK (DP purgée)</v>
+      <c r="K14" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="15">
@@ -1259,40 +1175,34 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>HOUSSAIT</v>
+        <v>SAINT-MARTIN-DE-FRESSENGEAS</v>
       </c>
       <c r="C15" t="str">
-        <v>33930 VENDAYS</v>
+        <v>24800 ST-MARTIN</v>
       </c>
       <c r="D15" t="str">
-        <v>33</v>
-      </c>
-      <c r="E15">
-        <v>500</v>
+        <v>24</v>
+      </c>
+      <c r="E15" t="str">
+        <v>MISSAULT Patrick</v>
       </c>
       <c r="F15">
-        <v>2800</v>
+        <v>388</v>
       </c>
       <c r="G15">
-        <v>1135</v>
+        <v>2250</v>
       </c>
       <c r="H15">
-        <v>567500</v>
+        <v>257021</v>
       </c>
       <c r="I15">
-        <v>82</v>
-      </c>
-      <c r="J15">
-        <v>46535</v>
-      </c>
-      <c r="K15">
-        <v>3500</v>
-      </c>
-      <c r="L15" t="str">
+        <v>35230</v>
+      </c>
+      <c r="J15" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M15" t="str">
-        <v>URBA OK (PC obtenu)</v>
+      <c r="K15" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="16">
@@ -1300,40 +1210,34 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>SOULIGNAC</v>
+        <v>SAINT-AVIT-SAINT-NAZAIRE</v>
       </c>
       <c r="C16" t="str">
-        <v>33860 VAL-DE-LIVENNE</v>
+        <v>33220 ST-AVIT</v>
       </c>
       <c r="D16" t="str">
         <v>33</v>
       </c>
-      <c r="E16">
-        <v>521.6</v>
+      <c r="E16" t="str">
+        <v>MARTIN Eric</v>
       </c>
       <c r="F16">
-        <v>2900</v>
+        <v>337</v>
       </c>
       <c r="G16">
-        <v>1130</v>
+        <v>1955</v>
       </c>
       <c r="H16">
-        <v>589408</v>
+        <v>204281</v>
       </c>
       <c r="I16">
-        <v>82</v>
-      </c>
-      <c r="J16">
-        <v>48331</v>
-      </c>
-      <c r="K16">
-        <v>3700</v>
-      </c>
-      <c r="L16" t="str">
+        <v>30734</v>
+      </c>
+      <c r="J16" t="str">
         <v>PdB signée 20 ans</v>
       </c>
-      <c r="M16" t="str">
-        <v>URBA OK (PC obtenu)</v>
+      <c r="K16" t="str">
+        <v>URBA OK</v>
       </c>
     </row>
     <row r="17">
@@ -1341,7 +1245,7 @@
         <v>TOTAL</v>
       </c>
       <c r="B17" t="str">
-        <v>15 CENTRALES SOLAIRES</v>
+        <v>15 CENTRALES SOLAIRES (15 PROJETS)</v>
       </c>
       <c r="C17" t="str">
         <v>AQUITAINE / OCCITANIE</v>
@@ -1349,37 +1253,31 @@
       <c r="D17" t="str">
         <v>7 Dpts</v>
       </c>
-      <c r="E17">
-        <v>6240</v>
+      <c r="E17" t="str">
+        <v>15 Exploitants sécurisés</v>
       </c>
       <c r="F17">
-        <v>35800</v>
+        <v>6240.2</v>
       </c>
       <c r="G17">
-        <v>1125</v>
+        <v>36190</v>
       </c>
       <c r="H17">
-        <v>7036000</v>
+        <v>3698035</v>
       </c>
       <c r="I17">
-        <v>82</v>
-      </c>
-      <c r="J17">
         <v>569527</v>
       </c>
-      <c r="K17">
-        <v>44300</v>
-      </c>
-      <c r="L17" t="str">
+      <c r="J17" t="str">
         <v>100% Sécurisé</v>
       </c>
-      <c r="M17" t="str">
+      <c r="K17" t="str">
         <v>100% Purgé</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>